<commit_message>
Add better analysis of differences between assignments and protocols, add international availablity report, persist retired officials
</commit_message>
<xml_diff>
--- a/activityAnalysis/Appointments_to_database.xlsx
+++ b/activityAnalysis/Appointments_to_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rachaelnaphtal/Documents/JudgingAnalysis/activityAnalysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDC8553-8194-9C46-87DA-0EE56371CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85066DD1-0C40-1C49-AEB9-8739AD182DAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3040" yWindow="760" windowWidth="14420" windowHeight="17020" xr2:uid="{3DC34758-EE40-AE44-9218-4BCDC75CCCC4}"/>
+    <workbookView xWindow="3040" yWindow="760" windowWidth="14420" windowHeight="16860" xr2:uid="{3DC34758-EE40-AE44-9218-4BCDC75CCCC4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2306,7 +2306,7 @@
         <v>4</v>
       </c>
       <c r="E76">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -3286,7 +3286,7 @@
         <v>9</v>
       </c>
       <c r="E145">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146" spans="1:6">
@@ -3699,7 +3699,7 @@
         <v>11</v>
       </c>
       <c r="E175">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="176" spans="1:6" ht="15" customHeight="1">

</xml_diff>